<commit_message>
chore: daily pipeline outputs (2026-08-05)
</commit_message>
<xml_diff>
--- a/data/flat/model_ledgers/soccer-poisson-dc.xlsx
+++ b/data/flat/model_ledgers/soccer-poisson-dc.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Predictions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Predictions'!$A$1:$AJ$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Predictions'!$A$1:$AJ$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ10"/>
+  <dimension ref="A1:AJ22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1622,8 +1622,1292 @@
       <c r="AI10" s="2" t="inlineStr"/>
       <c r="AJ10" s="2" t="inlineStr"/>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>0dc3613c43be46c8</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>401886532</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>0.480757</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>0.8699609882964889</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>-0.38920398829648895</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T15:00:54.071189Z</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T18:00Z</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="inlineStr"/>
+      <c r="W11" s="2" t="inlineStr"/>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr"/>
+      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AA11" s="2" t="inlineStr"/>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr"/>
+      <c r="AD11" s="2" t="inlineStr"/>
+      <c r="AE11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="inlineStr"/>
+      <c r="AG11" s="2" t="inlineStr"/>
+      <c r="AH11" s="2" t="inlineStr"/>
+      <c r="AI11" s="2" t="inlineStr"/>
+      <c r="AJ11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>c6dca9a2e2f4407f</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>401886532</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>0.480757</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>0.8599439775910364</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>-0.37918697759103637</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T16:50:24.939028Z</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T18:00Z</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="2" t="inlineStr"/>
+      <c r="W12" s="2" t="inlineStr"/>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="AA12" s="2" t="inlineStr"/>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>0.1629</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T21:59:03.837990Z</t>
+        </is>
+      </c>
+      <c r="AD12" s="2" t="inlineStr"/>
+      <c r="AE12" s="2" t="inlineStr"/>
+      <c r="AF12" s="2" t="inlineStr"/>
+      <c r="AG12" s="2" t="inlineStr"/>
+      <c r="AH12" s="2" t="inlineStr"/>
+      <c r="AI12" s="2" t="inlineStr"/>
+      <c r="AJ12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>81b4bca1acb44f5c</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>401841460</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>0.500109</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>0.4608294930875576</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>0.03927950691244242</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:23:20.586018Z</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T22:00Z</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="2" t="inlineStr"/>
+      <c r="W13" s="2" t="inlineStr"/>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr"/>
+      <c r="Z13" s="2" t="inlineStr"/>
+      <c r="AA13" s="2" t="inlineStr"/>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AD13" s="2" t="inlineStr"/>
+      <c r="AE13" s="2" t="inlineStr"/>
+      <c r="AF13" s="2" t="inlineStr"/>
+      <c r="AG13" s="2" t="inlineStr"/>
+      <c r="AH13" s="2" t="inlineStr"/>
+      <c r="AI13" s="2" t="inlineStr"/>
+      <c r="AJ13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>aa3c5ecea2a044dd</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>401843981</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>0.33003300330033003</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>0.12610199669966998</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:23:25.867092Z</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:00Z</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="2" t="inlineStr"/>
+      <c r="W14" s="2" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="AA14" s="2" t="inlineStr"/>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr"/>
+      <c r="AD14" s="2" t="inlineStr"/>
+      <c r="AE14" s="2" t="inlineStr"/>
+      <c r="AF14" s="2" t="inlineStr"/>
+      <c r="AG14" s="2" t="inlineStr"/>
+      <c r="AH14" s="2" t="inlineStr"/>
+      <c r="AI14" s="2" t="inlineStr"/>
+      <c r="AJ14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>777349270e5247f9</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>401843990</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>0.440521</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>0.4608294930875576</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>-0.02030849308755761</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:23:21.640701Z</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T23:00Z</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="inlineStr"/>
+      <c r="W15" s="2" t="inlineStr"/>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="AA15" s="2" t="inlineStr"/>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AD15" s="2" t="inlineStr"/>
+      <c r="AE15" s="2" t="inlineStr"/>
+      <c r="AF15" s="2" t="inlineStr"/>
+      <c r="AG15" s="2" t="inlineStr"/>
+      <c r="AH15" s="2" t="inlineStr"/>
+      <c r="AI15" s="2" t="inlineStr"/>
+      <c r="AJ15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>dd6a4559d28d4e8a</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>401871494</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>0.483062</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>0.3003003003003003</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>0.1827616996996997</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:23:23.018456Z</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:30Z</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr"/>
+      <c r="V16" s="2" t="inlineStr"/>
+      <c r="W16" s="2" t="inlineStr"/>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="AA16" s="2" t="inlineStr"/>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr"/>
+      <c r="AD16" s="2" t="inlineStr"/>
+      <c r="AE16" s="2" t="inlineStr"/>
+      <c r="AF16" s="2" t="inlineStr"/>
+      <c r="AG16" s="2" t="inlineStr"/>
+      <c r="AH16" s="2" t="inlineStr"/>
+      <c r="AI16" s="2" t="inlineStr"/>
+      <c r="AJ16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>360c0ad121a5407d</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>401867142</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>0.615056</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>0.7701149425287357</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>-0.15505894252873564</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:23:24.108314Z</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:30Z</t>
+        </is>
+      </c>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="2" t="inlineStr"/>
+      <c r="W17" s="2" t="inlineStr"/>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr"/>
+      <c r="Z17" s="2" t="inlineStr"/>
+      <c r="AA17" s="2" t="inlineStr"/>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr"/>
+      <c r="AD17" s="2" t="inlineStr"/>
+      <c r="AE17" s="2" t="inlineStr"/>
+      <c r="AF17" s="2" t="inlineStr"/>
+      <c r="AG17" s="2" t="inlineStr"/>
+      <c r="AH17" s="2" t="inlineStr"/>
+      <c r="AI17" s="2" t="inlineStr"/>
+      <c r="AJ17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>bba9580763d6485d</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>401841460</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>0.500109</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>0.4608294930875576</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>0.03927950691244242</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:34:06.752018Z</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T22:00Z</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="2" t="inlineStr"/>
+      <c r="W18" s="2" t="inlineStr"/>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr"/>
+      <c r="Z18" s="2" t="inlineStr"/>
+      <c r="AA18" s="2" t="inlineStr"/>
+      <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AD18" s="2" t="inlineStr"/>
+      <c r="AE18" s="2" t="inlineStr"/>
+      <c r="AF18" s="2" t="inlineStr"/>
+      <c r="AG18" s="2" t="inlineStr"/>
+      <c r="AH18" s="2" t="inlineStr"/>
+      <c r="AI18" s="2" t="inlineStr"/>
+      <c r="AJ18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>b5e72bec6e014f71</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>401843981</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>0.33003300330033003</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>0.12610199669966998</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:34:07.208609Z</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:00Z</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr"/>
+      <c r="V19" s="2" t="inlineStr"/>
+      <c r="W19" s="2" t="inlineStr"/>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y19" s="2" t="inlineStr"/>
+      <c r="Z19" s="2" t="inlineStr"/>
+      <c r="AA19" s="2" t="inlineStr"/>
+      <c r="AB19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AD19" s="2" t="inlineStr"/>
+      <c r="AE19" s="2" t="inlineStr"/>
+      <c r="AF19" s="2" t="inlineStr"/>
+      <c r="AG19" s="2" t="inlineStr"/>
+      <c r="AH19" s="2" t="inlineStr"/>
+      <c r="AI19" s="2" t="inlineStr"/>
+      <c r="AJ19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>51aea01a60e04a99</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>401843990</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>0.440521</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>0.4608294930875576</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>-0.02030849308755761</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:34:07.511498Z</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T23:00Z</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr"/>
+      <c r="V20" s="2" t="inlineStr"/>
+      <c r="W20" s="2" t="inlineStr"/>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr"/>
+      <c r="Z20" s="2" t="inlineStr"/>
+      <c r="AA20" s="2" t="inlineStr"/>
+      <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="inlineStr"/>
+      <c r="AE20" s="2" t="inlineStr"/>
+      <c r="AF20" s="2" t="inlineStr"/>
+      <c r="AG20" s="2" t="inlineStr"/>
+      <c r="AH20" s="2" t="inlineStr"/>
+      <c r="AI20" s="2" t="inlineStr"/>
+      <c r="AJ20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>16df25b9f6774861</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>401871494</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>0.483062</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>0.3003003003003003</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>0.1827616996996997</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:34:08.269054Z</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:30Z</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr"/>
+      <c r="V21" s="2" t="inlineStr"/>
+      <c r="W21" s="2" t="inlineStr"/>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr"/>
+      <c r="Z21" s="2" t="inlineStr"/>
+      <c r="AA21" s="2" t="inlineStr"/>
+      <c r="AB21" s="2" t="inlineStr"/>
+      <c r="AC21" s="2" t="inlineStr"/>
+      <c r="AD21" s="2" t="inlineStr"/>
+      <c r="AE21" s="2" t="inlineStr"/>
+      <c r="AF21" s="2" t="inlineStr"/>
+      <c r="AG21" s="2" t="inlineStr"/>
+      <c r="AH21" s="2" t="inlineStr"/>
+      <c r="AI21" s="2" t="inlineStr"/>
+      <c r="AJ21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>b3c3319a44ce48de</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>401867142</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>0.615056</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>0.7297297297297298</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>-0.11467372972972978</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T04:34:09.148998Z</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:30Z</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr"/>
+      <c r="V22" s="2" t="inlineStr"/>
+      <c r="W22" s="2" t="inlineStr"/>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr"/>
+      <c r="AA22" s="2" t="inlineStr"/>
+      <c r="AB22" s="2" t="inlineStr"/>
+      <c r="AC22" s="2" t="inlineStr"/>
+      <c r="AD22" s="2" t="inlineStr"/>
+      <c r="AE22" s="2" t="inlineStr"/>
+      <c r="AF22" s="2" t="inlineStr"/>
+      <c r="AG22" s="2" t="inlineStr"/>
+      <c r="AH22" s="2" t="inlineStr"/>
+      <c r="AI22" s="2" t="inlineStr"/>
+      <c r="AJ22" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ10"/>
+  <autoFilter ref="A1:AJ22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(data): sync daily pipeline outputs and baseline refreshes
Routine ingestion sync: odds snapshots, MLB/WNBA availability data,
ESPN scoreboard raw pulls (2026-07-03 through 2026-08-07), model
ledgers, and rebuild parquet/db state. Also picks up the latest
MLB baseline refresh (park factors recomputed on 7835 games through
2026-08-05, relief ERA updated) and esports/KBO/NPB elo config updates.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flat/model_ledgers/soccer-poisson-dc.xlsx
+++ b/data/flat/model_ledgers/soccer-poisson-dc.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Predictions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Predictions'!$A$1:$AJ$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Predictions'!$A$1:$AJ$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ37"/>
+  <dimension ref="A1:AJ63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4508,8 +4508,2836 @@
       <c r="AI37" s="2" t="inlineStr"/>
       <c r="AJ37" s="2" t="inlineStr"/>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>9e28e8f3e6ff46c2</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>401841460</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>0.500109</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>0.4608294930875576</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>0.03927950691244242</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T17:01:54.470179Z</t>
+        </is>
+      </c>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T22:00Z</t>
+        </is>
+      </c>
+      <c r="T38" s="2" t="inlineStr"/>
+      <c r="U38" s="2" t="inlineStr"/>
+      <c r="V38" s="2" t="inlineStr"/>
+      <c r="W38" s="2" t="inlineStr"/>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y38" s="2" t="inlineStr"/>
+      <c r="Z38" s="2" t="inlineStr"/>
+      <c r="AA38" s="2" t="inlineStr"/>
+      <c r="AB38" s="2" t="inlineStr"/>
+      <c r="AC38" s="2" t="inlineStr"/>
+      <c r="AD38" s="2" t="inlineStr"/>
+      <c r="AE38" s="2" t="inlineStr"/>
+      <c r="AF38" s="2" t="inlineStr"/>
+      <c r="AG38" s="2" t="inlineStr"/>
+      <c r="AH38" s="2" t="inlineStr"/>
+      <c r="AI38" s="2" t="inlineStr"/>
+      <c r="AJ38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>b702d801c5c1411b</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>401843981</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>0.33003300330033003</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>0.12610199669966998</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T17:01:54.694147Z</t>
+        </is>
+      </c>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:00Z</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="inlineStr"/>
+      <c r="U39" s="2" t="inlineStr"/>
+      <c r="V39" s="2" t="inlineStr"/>
+      <c r="W39" s="2" t="inlineStr"/>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="Y39" s="2" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="Z39" s="2" t="inlineStr"/>
+      <c r="AA39" s="2" t="inlineStr"/>
+      <c r="AB39" s="2" t="inlineStr">
+        <is>
+          <t>-0.0000</t>
+        </is>
+      </c>
+      <c r="AC39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06T00:20:47.940777Z</t>
+        </is>
+      </c>
+      <c r="AD39" s="2" t="inlineStr"/>
+      <c r="AE39" s="2" t="inlineStr"/>
+      <c r="AF39" s="2" t="inlineStr"/>
+      <c r="AG39" s="2" t="inlineStr"/>
+      <c r="AH39" s="2" t="inlineStr"/>
+      <c r="AI39" s="2" t="inlineStr"/>
+      <c r="AJ39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>7eb90b44e90d4c0c</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>401843990</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>0.440521</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>0.4608294930875576</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>-0.02030849308755761</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T17:01:54.741392Z</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T22:00Z</t>
+        </is>
+      </c>
+      <c r="T40" s="2" t="inlineStr"/>
+      <c r="U40" s="2" t="inlineStr"/>
+      <c r="V40" s="2" t="inlineStr"/>
+      <c r="W40" s="2" t="inlineStr"/>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y40" s="2" t="inlineStr"/>
+      <c r="Z40" s="2" t="inlineStr"/>
+      <c r="AA40" s="2" t="inlineStr"/>
+      <c r="AB40" s="2" t="inlineStr"/>
+      <c r="AC40" s="2" t="inlineStr"/>
+      <c r="AD40" s="2" t="inlineStr"/>
+      <c r="AE40" s="2" t="inlineStr"/>
+      <c r="AF40" s="2" t="inlineStr"/>
+      <c r="AG40" s="2" t="inlineStr"/>
+      <c r="AH40" s="2" t="inlineStr"/>
+      <c r="AI40" s="2" t="inlineStr"/>
+      <c r="AJ40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>e234724110c64831</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>401867142</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>0.615056</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>0.6598639455782314</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>-0.04480794557823131</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T17:01:55.596249Z</t>
+        </is>
+      </c>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T18:30Z</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr"/>
+      <c r="U41" s="2" t="inlineStr"/>
+      <c r="V41" s="2" t="inlineStr"/>
+      <c r="W41" s="2" t="inlineStr"/>
+      <c r="X41" s="2" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="Y41" s="2" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="AA41" s="2" t="inlineStr"/>
+      <c r="AB41" s="2" t="inlineStr">
+        <is>
+          <t>-0.0000</t>
+        </is>
+      </c>
+      <c r="AC41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T20:58:28.992396Z</t>
+        </is>
+      </c>
+      <c r="AD41" s="2" t="inlineStr"/>
+      <c r="AE41" s="2" t="inlineStr"/>
+      <c r="AF41" s="2" t="inlineStr"/>
+      <c r="AG41" s="2" t="inlineStr"/>
+      <c r="AH41" s="2" t="inlineStr"/>
+      <c r="AI41" s="2" t="inlineStr"/>
+      <c r="AJ41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>f57c437d70f744b6</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>401886451</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>0.526434</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>0.49019607843137253</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>0.03623792156862743</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T17:01:55.733913Z</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T19:00Z</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr"/>
+      <c r="U42" s="2" t="inlineStr"/>
+      <c r="V42" s="2" t="inlineStr"/>
+      <c r="W42" s="2" t="inlineStr"/>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="Y42" s="2" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="Z42" s="2" t="inlineStr"/>
+      <c r="AA42" s="2" t="inlineStr"/>
+      <c r="AB42" s="2" t="inlineStr">
+        <is>
+          <t>-0.0000</t>
+        </is>
+      </c>
+      <c r="AC42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T20:58:29.516536Z</t>
+        </is>
+      </c>
+      <c r="AD42" s="2" t="inlineStr"/>
+      <c r="AE42" s="2" t="inlineStr"/>
+      <c r="AF42" s="2" t="inlineStr"/>
+      <c r="AG42" s="2" t="inlineStr"/>
+      <c r="AH42" s="2" t="inlineStr"/>
+      <c r="AI42" s="2" t="inlineStr"/>
+      <c r="AJ42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>91fa12815d134861</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>401841460</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>0.500109</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>0.5192307692307692</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr"/>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>-0.019121769230769137</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T21:00:53.073019Z</t>
+        </is>
+      </c>
+      <c r="S43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T22:00Z</t>
+        </is>
+      </c>
+      <c r="T43" s="2" t="inlineStr"/>
+      <c r="U43" s="2" t="inlineStr"/>
+      <c r="V43" s="2" t="inlineStr"/>
+      <c r="W43" s="2" t="inlineStr"/>
+      <c r="X43" s="2" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="Y43" s="2" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="AA43" s="2" t="inlineStr"/>
+      <c r="AB43" s="2" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="AC43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06T00:20:48.762339Z</t>
+        </is>
+      </c>
+      <c r="AD43" s="2" t="inlineStr"/>
+      <c r="AE43" s="2" t="inlineStr"/>
+      <c r="AF43" s="2" t="inlineStr"/>
+      <c r="AG43" s="2" t="inlineStr"/>
+      <c r="AH43" s="2" t="inlineStr"/>
+      <c r="AI43" s="2" t="inlineStr"/>
+      <c r="AJ43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>af4c45df932c43c6</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>401843990</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>0.440521</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>0.4608294930875576</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr"/>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>-0.02030849308755761</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T21:00:53.307981Z</t>
+        </is>
+      </c>
+      <c r="S44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T22:00Z</t>
+        </is>
+      </c>
+      <c r="T44" s="2" t="inlineStr"/>
+      <c r="U44" s="2" t="inlineStr"/>
+      <c r="V44" s="2" t="inlineStr"/>
+      <c r="W44" s="2" t="inlineStr"/>
+      <c r="X44" s="2" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="Y44" s="2" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="Z44" s="2" t="inlineStr"/>
+      <c r="AA44" s="2" t="inlineStr"/>
+      <c r="AB44" s="2" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="AC44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06T03:26:39.209741Z</t>
+        </is>
+      </c>
+      <c r="AD44" s="2" t="inlineStr"/>
+      <c r="AE44" s="2" t="inlineStr"/>
+      <c r="AF44" s="2" t="inlineStr"/>
+      <c r="AG44" s="2" t="inlineStr"/>
+      <c r="AH44" s="2" t="inlineStr"/>
+      <c r="AI44" s="2" t="inlineStr"/>
+      <c r="AJ44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>e929ef9f2186404b</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>401860269</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>0.483295</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>0.6996996996996997</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr"/>
+      <c r="Q45" s="2" t="inlineStr">
+        <is>
+          <t>-0.21640469969969972</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T06:02:30.231228Z</t>
+        </is>
+      </c>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T23:30Z</t>
+        </is>
+      </c>
+      <c r="T45" s="2" t="inlineStr"/>
+      <c r="U45" s="2" t="inlineStr"/>
+      <c r="V45" s="2" t="inlineStr"/>
+      <c r="W45" s="2" t="inlineStr"/>
+      <c r="X45" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y45" s="2" t="inlineStr"/>
+      <c r="Z45" s="2" t="inlineStr"/>
+      <c r="AA45" s="2" t="inlineStr"/>
+      <c r="AB45" s="2" t="inlineStr"/>
+      <c r="AC45" s="2" t="inlineStr"/>
+      <c r="AD45" s="2" t="inlineStr"/>
+      <c r="AE45" s="2" t="inlineStr"/>
+      <c r="AF45" s="2" t="inlineStr"/>
+      <c r="AG45" s="2" t="inlineStr"/>
+      <c r="AH45" s="2" t="inlineStr"/>
+      <c r="AI45" s="2" t="inlineStr"/>
+      <c r="AJ45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>0fa8a25029c942be</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>401841491</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>0.6598639455782314</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr"/>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>-0.20372894557823135</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T06:02:30.348619Z</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T22:30Z</t>
+        </is>
+      </c>
+      <c r="T46" s="2" t="inlineStr"/>
+      <c r="U46" s="2" t="inlineStr"/>
+      <c r="V46" s="2" t="inlineStr"/>
+      <c r="W46" s="2" t="inlineStr"/>
+      <c r="X46" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y46" s="2" t="inlineStr"/>
+      <c r="Z46" s="2" t="inlineStr"/>
+      <c r="AA46" s="2" t="inlineStr"/>
+      <c r="AB46" s="2" t="inlineStr"/>
+      <c r="AC46" s="2" t="inlineStr"/>
+      <c r="AD46" s="2" t="inlineStr"/>
+      <c r="AE46" s="2" t="inlineStr"/>
+      <c r="AF46" s="2" t="inlineStr"/>
+      <c r="AG46" s="2" t="inlineStr"/>
+      <c r="AH46" s="2" t="inlineStr"/>
+      <c r="AI46" s="2" t="inlineStr"/>
+      <c r="AJ46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>df8f6ef3dc17469d</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>401905201</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>0.34965034965034963</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="inlineStr"/>
+      <c r="Q47" s="2" t="inlineStr">
+        <is>
+          <t>0.10648465034965038</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T06:02:30.762429Z</t>
+        </is>
+      </c>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T22:00Z</t>
+        </is>
+      </c>
+      <c r="T47" s="2" t="inlineStr"/>
+      <c r="U47" s="2" t="inlineStr"/>
+      <c r="V47" s="2" t="inlineStr"/>
+      <c r="W47" s="2" t="inlineStr"/>
+      <c r="X47" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y47" s="2" t="inlineStr"/>
+      <c r="Z47" s="2" t="inlineStr"/>
+      <c r="AA47" s="2" t="inlineStr"/>
+      <c r="AB47" s="2" t="inlineStr"/>
+      <c r="AC47" s="2" t="inlineStr"/>
+      <c r="AD47" s="2" t="inlineStr"/>
+      <c r="AE47" s="2" t="inlineStr"/>
+      <c r="AF47" s="2" t="inlineStr"/>
+      <c r="AG47" s="2" t="inlineStr"/>
+      <c r="AH47" s="2" t="inlineStr"/>
+      <c r="AI47" s="2" t="inlineStr"/>
+      <c r="AJ47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>dbff0113a09d49d5</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>401886111</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>0.394611</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>0.3597122302158273</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr"/>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>0.03489876978417267</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T06:02:31.165683Z</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T20:15Z</t>
+        </is>
+      </c>
+      <c r="T48" s="2" t="inlineStr"/>
+      <c r="U48" s="2" t="inlineStr"/>
+      <c r="V48" s="2" t="inlineStr"/>
+      <c r="W48" s="2" t="inlineStr"/>
+      <c r="X48" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y48" s="2" t="inlineStr"/>
+      <c r="Z48" s="2" t="inlineStr"/>
+      <c r="AA48" s="2" t="inlineStr"/>
+      <c r="AB48" s="2" t="inlineStr"/>
+      <c r="AC48" s="2" t="inlineStr"/>
+      <c r="AD48" s="2" t="inlineStr"/>
+      <c r="AE48" s="2" t="inlineStr"/>
+      <c r="AF48" s="2" t="inlineStr"/>
+      <c r="AG48" s="2" t="inlineStr"/>
+      <c r="AH48" s="2" t="inlineStr"/>
+      <c r="AI48" s="2" t="inlineStr"/>
+      <c r="AJ48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>b7de51662e2440d5</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>401867952</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>0.784326</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>0.5391705069124424</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr"/>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>0.24515549308755757</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T06:02:31.343362Z</t>
+        </is>
+      </c>
+      <c r="S49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T12:00Z</t>
+        </is>
+      </c>
+      <c r="T49" s="2" t="inlineStr"/>
+      <c r="U49" s="2" t="inlineStr"/>
+      <c r="V49" s="2" t="inlineStr"/>
+      <c r="W49" s="2" t="inlineStr"/>
+      <c r="X49" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y49" s="2" t="inlineStr"/>
+      <c r="Z49" s="2" t="inlineStr"/>
+      <c r="AA49" s="2" t="inlineStr"/>
+      <c r="AB49" s="2" t="inlineStr"/>
+      <c r="AC49" s="2" t="inlineStr"/>
+      <c r="AD49" s="2" t="inlineStr"/>
+      <c r="AE49" s="2" t="inlineStr"/>
+      <c r="AF49" s="2" t="inlineStr"/>
+      <c r="AG49" s="2" t="inlineStr"/>
+      <c r="AH49" s="2" t="inlineStr"/>
+      <c r="AI49" s="2" t="inlineStr"/>
+      <c r="AJ49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>c2476d75b74c4589</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>401860269</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>0.483295</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>0.6996996996996997</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr"/>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>-0.21640469969969972</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T09:08:45.801754Z</t>
+        </is>
+      </c>
+      <c r="S50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T23:30Z</t>
+        </is>
+      </c>
+      <c r="T50" s="2" t="inlineStr"/>
+      <c r="U50" s="2" t="inlineStr"/>
+      <c r="V50" s="2" t="inlineStr"/>
+      <c r="W50" s="2" t="inlineStr"/>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y50" s="2" t="inlineStr"/>
+      <c r="Z50" s="2" t="inlineStr"/>
+      <c r="AA50" s="2" t="inlineStr"/>
+      <c r="AB50" s="2" t="inlineStr"/>
+      <c r="AC50" s="2" t="inlineStr"/>
+      <c r="AD50" s="2" t="inlineStr"/>
+      <c r="AE50" s="2" t="inlineStr"/>
+      <c r="AF50" s="2" t="inlineStr"/>
+      <c r="AG50" s="2" t="inlineStr"/>
+      <c r="AH50" s="2" t="inlineStr"/>
+      <c r="AI50" s="2" t="inlineStr"/>
+      <c r="AJ50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>c1103e9137f84dad</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>401841491</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>0.6598639455782314</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr"/>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>-0.20372894557823135</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T09:08:45.867163Z</t>
+        </is>
+      </c>
+      <c r="S51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T22:30Z</t>
+        </is>
+      </c>
+      <c r="T51" s="2" t="inlineStr"/>
+      <c r="U51" s="2" t="inlineStr"/>
+      <c r="V51" s="2" t="inlineStr"/>
+      <c r="W51" s="2" t="inlineStr"/>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y51" s="2" t="inlineStr"/>
+      <c r="Z51" s="2" t="inlineStr"/>
+      <c r="AA51" s="2" t="inlineStr"/>
+      <c r="AB51" s="2" t="inlineStr"/>
+      <c r="AC51" s="2" t="inlineStr"/>
+      <c r="AD51" s="2" t="inlineStr"/>
+      <c r="AE51" s="2" t="inlineStr"/>
+      <c r="AF51" s="2" t="inlineStr"/>
+      <c r="AG51" s="2" t="inlineStr"/>
+      <c r="AH51" s="2" t="inlineStr"/>
+      <c r="AI51" s="2" t="inlineStr"/>
+      <c r="AJ51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>e0c9b04eb32c4e67</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>401905201</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>0.34965034965034963</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr"/>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>0.10648465034965038</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T09:08:46.407563Z</t>
+        </is>
+      </c>
+      <c r="S52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T22:00Z</t>
+        </is>
+      </c>
+      <c r="T52" s="2" t="inlineStr"/>
+      <c r="U52" s="2" t="inlineStr"/>
+      <c r="V52" s="2" t="inlineStr"/>
+      <c r="W52" s="2" t="inlineStr"/>
+      <c r="X52" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y52" s="2" t="inlineStr"/>
+      <c r="Z52" s="2" t="inlineStr"/>
+      <c r="AA52" s="2" t="inlineStr"/>
+      <c r="AB52" s="2" t="inlineStr"/>
+      <c r="AC52" s="2" t="inlineStr"/>
+      <c r="AD52" s="2" t="inlineStr"/>
+      <c r="AE52" s="2" t="inlineStr"/>
+      <c r="AF52" s="2" t="inlineStr"/>
+      <c r="AG52" s="2" t="inlineStr"/>
+      <c r="AH52" s="2" t="inlineStr"/>
+      <c r="AI52" s="2" t="inlineStr"/>
+      <c r="AJ52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>241b4361d84f41c4</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>401886111</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr"/>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>0.394611</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr"/>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>0.3597122302158273</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="inlineStr"/>
+      <c r="Q53" s="2" t="inlineStr">
+        <is>
+          <t>0.03489876978417267</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T09:08:46.908185Z</t>
+        </is>
+      </c>
+      <c r="S53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T20:15Z</t>
+        </is>
+      </c>
+      <c r="T53" s="2" t="inlineStr"/>
+      <c r="U53" s="2" t="inlineStr"/>
+      <c r="V53" s="2" t="inlineStr"/>
+      <c r="W53" s="2" t="inlineStr"/>
+      <c r="X53" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y53" s="2" t="inlineStr"/>
+      <c r="Z53" s="2" t="inlineStr"/>
+      <c r="AA53" s="2" t="inlineStr"/>
+      <c r="AB53" s="2" t="inlineStr"/>
+      <c r="AC53" s="2" t="inlineStr"/>
+      <c r="AD53" s="2" t="inlineStr"/>
+      <c r="AE53" s="2" t="inlineStr"/>
+      <c r="AF53" s="2" t="inlineStr"/>
+      <c r="AG53" s="2" t="inlineStr"/>
+      <c r="AH53" s="2" t="inlineStr"/>
+      <c r="AI53" s="2" t="inlineStr"/>
+      <c r="AJ53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>5594bf45e1bb46d4</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>401867952</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>0.784326</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>0.5192307692307692</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>0.2650952307692308</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T09:08:46.980092Z</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T12:00Z</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr"/>
+      <c r="U54" s="2" t="inlineStr"/>
+      <c r="V54" s="2" t="inlineStr"/>
+      <c r="W54" s="2" t="inlineStr"/>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="Y54" s="2" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="Z54" s="2" t="inlineStr"/>
+      <c r="AA54" s="2" t="inlineStr"/>
+      <c r="AB54" s="2" t="inlineStr">
+        <is>
+          <t>1.8519</t>
+        </is>
+      </c>
+      <c r="AC54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T15:18:26.196646Z</t>
+        </is>
+      </c>
+      <c r="AD54" s="2" t="inlineStr"/>
+      <c r="AE54" s="2" t="inlineStr"/>
+      <c r="AF54" s="2" t="inlineStr"/>
+      <c r="AG54" s="2" t="inlineStr"/>
+      <c r="AH54" s="2" t="inlineStr"/>
+      <c r="AI54" s="2" t="inlineStr"/>
+      <c r="AJ54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>f4ca737283634db2</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>401860269</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr"/>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>0.483295</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>0.6996996996996997</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr"/>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>-0.21640469969969972</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T12:14:46.828297Z</t>
+        </is>
+      </c>
+      <c r="S55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T23:30Z</t>
+        </is>
+      </c>
+      <c r="T55" s="2" t="inlineStr"/>
+      <c r="U55" s="2" t="inlineStr"/>
+      <c r="V55" s="2" t="inlineStr"/>
+      <c r="W55" s="2" t="inlineStr"/>
+      <c r="X55" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y55" s="2" t="inlineStr"/>
+      <c r="Z55" s="2" t="inlineStr"/>
+      <c r="AA55" s="2" t="inlineStr"/>
+      <c r="AB55" s="2" t="inlineStr"/>
+      <c r="AC55" s="2" t="inlineStr"/>
+      <c r="AD55" s="2" t="inlineStr"/>
+      <c r="AE55" s="2" t="inlineStr"/>
+      <c r="AF55" s="2" t="inlineStr"/>
+      <c r="AG55" s="2" t="inlineStr"/>
+      <c r="AH55" s="2" t="inlineStr"/>
+      <c r="AI55" s="2" t="inlineStr"/>
+      <c r="AJ55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>5abdbc380fac4ad0</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>401841491</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>0.6503496503496503</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr"/>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>-0.1942146503496503</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T12:14:46.896697Z</t>
+        </is>
+      </c>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T22:30Z</t>
+        </is>
+      </c>
+      <c r="T56" s="2" t="inlineStr"/>
+      <c r="U56" s="2" t="inlineStr"/>
+      <c r="V56" s="2" t="inlineStr"/>
+      <c r="W56" s="2" t="inlineStr"/>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y56" s="2" t="inlineStr"/>
+      <c r="Z56" s="2" t="inlineStr"/>
+      <c r="AA56" s="2" t="inlineStr"/>
+      <c r="AB56" s="2" t="inlineStr"/>
+      <c r="AC56" s="2" t="inlineStr"/>
+      <c r="AD56" s="2" t="inlineStr"/>
+      <c r="AE56" s="2" t="inlineStr"/>
+      <c r="AF56" s="2" t="inlineStr"/>
+      <c r="AG56" s="2" t="inlineStr"/>
+      <c r="AH56" s="2" t="inlineStr"/>
+      <c r="AI56" s="2" t="inlineStr"/>
+      <c r="AJ56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>237715fa7d474ec5</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>401905201</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>0.3597122302158273</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr"/>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>0.09642276978417269</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T12:14:47.384433Z</t>
+        </is>
+      </c>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T22:00Z</t>
+        </is>
+      </c>
+      <c r="T57" s="2" t="inlineStr"/>
+      <c r="U57" s="2" t="inlineStr"/>
+      <c r="V57" s="2" t="inlineStr"/>
+      <c r="W57" s="2" t="inlineStr"/>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y57" s="2" t="inlineStr"/>
+      <c r="Z57" s="2" t="inlineStr"/>
+      <c r="AA57" s="2" t="inlineStr"/>
+      <c r="AB57" s="2" t="inlineStr"/>
+      <c r="AC57" s="2" t="inlineStr"/>
+      <c r="AD57" s="2" t="inlineStr"/>
+      <c r="AE57" s="2" t="inlineStr"/>
+      <c r="AF57" s="2" t="inlineStr"/>
+      <c r="AG57" s="2" t="inlineStr"/>
+      <c r="AH57" s="2" t="inlineStr"/>
+      <c r="AI57" s="2" t="inlineStr"/>
+      <c r="AJ57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>766916954f4a4afe</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>401886111</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>0.394611</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>0.37037037037037035</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr"/>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>0.02424062962962964</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T12:14:47.703094Z</t>
+        </is>
+      </c>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T20:15Z</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="inlineStr"/>
+      <c r="U58" s="2" t="inlineStr"/>
+      <c r="V58" s="2" t="inlineStr"/>
+      <c r="W58" s="2" t="inlineStr"/>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y58" s="2" t="inlineStr"/>
+      <c r="Z58" s="2" t="inlineStr"/>
+      <c r="AA58" s="2" t="inlineStr"/>
+      <c r="AB58" s="2" t="inlineStr"/>
+      <c r="AC58" s="2" t="inlineStr"/>
+      <c r="AD58" s="2" t="inlineStr"/>
+      <c r="AE58" s="2" t="inlineStr"/>
+      <c r="AF58" s="2" t="inlineStr"/>
+      <c r="AG58" s="2" t="inlineStr"/>
+      <c r="AH58" s="2" t="inlineStr"/>
+      <c r="AI58" s="2" t="inlineStr"/>
+      <c r="AJ58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>f34aaf95d2784612</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>401860269</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>0.483295</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>0.6996996996996997</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr"/>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>-0.21640469969969972</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T15:20:40.774058Z</t>
+        </is>
+      </c>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T23:30Z</t>
+        </is>
+      </c>
+      <c r="T59" s="2" t="inlineStr"/>
+      <c r="U59" s="2" t="inlineStr"/>
+      <c r="V59" s="2" t="inlineStr"/>
+      <c r="W59" s="2" t="inlineStr"/>
+      <c r="X59" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y59" s="2" t="inlineStr"/>
+      <c r="Z59" s="2" t="inlineStr"/>
+      <c r="AA59" s="2" t="inlineStr"/>
+      <c r="AB59" s="2" t="inlineStr"/>
+      <c r="AC59" s="2" t="inlineStr"/>
+      <c r="AD59" s="2" t="inlineStr"/>
+      <c r="AE59" s="2" t="inlineStr"/>
+      <c r="AF59" s="2" t="inlineStr"/>
+      <c r="AG59" s="2" t="inlineStr"/>
+      <c r="AH59" s="2" t="inlineStr"/>
+      <c r="AI59" s="2" t="inlineStr"/>
+      <c r="AJ59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>e123fbca024b4a60</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>401841491</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>0.6503496503496503</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr"/>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>-0.1942146503496503</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T15:20:40.891696Z</t>
+        </is>
+      </c>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T22:30Z</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr"/>
+      <c r="U60" s="2" t="inlineStr"/>
+      <c r="V60" s="2" t="inlineStr"/>
+      <c r="W60" s="2" t="inlineStr"/>
+      <c r="X60" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y60" s="2" t="inlineStr"/>
+      <c r="Z60" s="2" t="inlineStr"/>
+      <c r="AA60" s="2" t="inlineStr"/>
+      <c r="AB60" s="2" t="inlineStr"/>
+      <c r="AC60" s="2" t="inlineStr"/>
+      <c r="AD60" s="2" t="inlineStr"/>
+      <c r="AE60" s="2" t="inlineStr"/>
+      <c r="AF60" s="2" t="inlineStr"/>
+      <c r="AG60" s="2" t="inlineStr"/>
+      <c r="AH60" s="2" t="inlineStr"/>
+      <c r="AI60" s="2" t="inlineStr"/>
+      <c r="AJ60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>6522aaa12dc1429c</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>401905201</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>0.456135</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>0.33003300330033003</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr"/>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>0.12610199669966998</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T15:20:41.371011Z</t>
+        </is>
+      </c>
+      <c r="S61" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T22:00Z</t>
+        </is>
+      </c>
+      <c r="T61" s="2" t="inlineStr"/>
+      <c r="U61" s="2" t="inlineStr"/>
+      <c r="V61" s="2" t="inlineStr"/>
+      <c r="W61" s="2" t="inlineStr"/>
+      <c r="X61" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y61" s="2" t="inlineStr"/>
+      <c r="Z61" s="2" t="inlineStr"/>
+      <c r="AA61" s="2" t="inlineStr"/>
+      <c r="AB61" s="2" t="inlineStr"/>
+      <c r="AC61" s="2" t="inlineStr"/>
+      <c r="AD61" s="2" t="inlineStr"/>
+      <c r="AE61" s="2" t="inlineStr"/>
+      <c r="AF61" s="2" t="inlineStr"/>
+      <c r="AG61" s="2" t="inlineStr"/>
+      <c r="AH61" s="2" t="inlineStr"/>
+      <c r="AI61" s="2" t="inlineStr"/>
+      <c r="AJ61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>ff3bac53f4cb44fd</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>401886111</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>0.394611</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>0.390625</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr"/>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>0.0039859999999999896</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T15:20:41.859430Z</t>
+        </is>
+      </c>
+      <c r="S62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T20:15Z</t>
+        </is>
+      </c>
+      <c r="T62" s="2" t="inlineStr"/>
+      <c r="U62" s="2" t="inlineStr"/>
+      <c r="V62" s="2" t="inlineStr"/>
+      <c r="W62" s="2" t="inlineStr"/>
+      <c r="X62" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y62" s="2" t="inlineStr"/>
+      <c r="Z62" s="2" t="inlineStr"/>
+      <c r="AA62" s="2" t="inlineStr"/>
+      <c r="AB62" s="2" t="inlineStr"/>
+      <c r="AC62" s="2" t="inlineStr"/>
+      <c r="AD62" s="2" t="inlineStr"/>
+      <c r="AE62" s="2" t="inlineStr"/>
+      <c r="AF62" s="2" t="inlineStr"/>
+      <c r="AG62" s="2" t="inlineStr"/>
+      <c r="AH62" s="2" t="inlineStr"/>
+      <c r="AI62" s="2" t="inlineStr"/>
+      <c r="AJ62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>efe721ecc7ca4b06</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>c95ec2023134439ab985cb4cdcc58243749b9deb564fca7a2d587c15c9875427</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>401906279</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>0.564448</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>0.1798561151079137</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr"/>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>0.3845918848920863</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T15:20:42.028691Z</t>
+        </is>
+      </c>
+      <c r="S63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:45Z</t>
+        </is>
+      </c>
+      <c r="T63" s="2" t="inlineStr"/>
+      <c r="U63" s="2" t="inlineStr"/>
+      <c r="V63" s="2" t="inlineStr"/>
+      <c r="W63" s="2" t="inlineStr"/>
+      <c r="X63" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y63" s="2" t="inlineStr"/>
+      <c r="Z63" s="2" t="inlineStr"/>
+      <c r="AA63" s="2" t="inlineStr"/>
+      <c r="AB63" s="2" t="inlineStr"/>
+      <c r="AC63" s="2" t="inlineStr"/>
+      <c r="AD63" s="2" t="inlineStr"/>
+      <c r="AE63" s="2" t="inlineStr"/>
+      <c r="AF63" s="2" t="inlineStr"/>
+      <c r="AG63" s="2" t="inlineStr"/>
+      <c r="AH63" s="2" t="inlineStr"/>
+      <c r="AI63" s="2" t="inlineStr"/>
+      <c r="AJ63" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ37"/>
+  <autoFilter ref="A1:AJ63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>